<commit_message>
Cash Operations Dashboard + Update
</commit_message>
<xml_diff>
--- a/Stock Selection/OPEN POSITION.xlsx
+++ b/Stock Selection/OPEN POSITION.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q107"/>
+  <dimension ref="A1:Q110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,7 +544,7 @@
         <v>15.3</v>
       </c>
       <c r="H2" t="n">
-        <v>21.3</v>
+        <v>20.97</v>
       </c>
       <c r="I2" t="n">
         <v>5.35</v>
@@ -564,7 +564,7 @@
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>2.09</v>
+        <v>1.98</v>
       </c>
       <c r="Q2" t="inlineStr"/>
     </row>
@@ -593,7 +593,7 @@
         <v>34.55</v>
       </c>
       <c r="H3" t="n">
-        <v>32.31</v>
+        <v>31.46</v>
       </c>
       <c r="I3" t="n">
         <v>10</v>
@@ -613,7 +613,7 @@
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>-0.65</v>
+        <v>-0.9</v>
       </c>
       <c r="Q3" t="inlineStr"/>
     </row>
@@ -642,7 +642,7 @@
         <v>16.425</v>
       </c>
       <c r="H4" t="n">
-        <v>15.394</v>
+        <v>15.382</v>
       </c>
       <c r="I4" t="n">
         <v>17.11</v>
@@ -662,7 +662,7 @@
         <v>0</v>
       </c>
       <c r="P4" t="n">
-        <v>0.24</v>
+        <v>0.17</v>
       </c>
       <c r="Q4" t="inlineStr"/>
     </row>
@@ -691,7 +691,7 @@
         <v>36.1</v>
       </c>
       <c r="H5" t="n">
-        <v>36.44</v>
+        <v>36.95</v>
       </c>
       <c r="I5" t="n">
         <v>10</v>
@@ -711,7 +711,7 @@
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>0.09</v>
+        <v>0.24</v>
       </c>
       <c r="Q5" t="inlineStr"/>
     </row>
@@ -740,7 +740,7 @@
         <v>165.35</v>
       </c>
       <c r="H6" t="n">
-        <v>197.55</v>
+        <v>196.05</v>
       </c>
       <c r="I6" t="n">
         <v>15</v>
@@ -760,7 +760,7 @@
         <v>0</v>
       </c>
       <c r="P6" t="n">
-        <v>2.92</v>
+        <v>2.78</v>
       </c>
       <c r="Q6" t="inlineStr"/>
     </row>
@@ -789,7 +789,7 @@
         <v>15.57</v>
       </c>
       <c r="H7" t="n">
-        <v>17.88</v>
+        <v>17.63</v>
       </c>
       <c r="I7" t="n">
         <v>10</v>
@@ -809,7 +809,7 @@
         <v>0</v>
       </c>
       <c r="P7" t="n">
-        <v>1.48</v>
+        <v>1.32</v>
       </c>
       <c r="Q7" t="inlineStr"/>
     </row>
@@ -838,7 +838,7 @@
         <v>21.85</v>
       </c>
       <c r="H8" t="n">
-        <v>17.3</v>
+        <v>17.17</v>
       </c>
       <c r="I8" t="n">
         <v>10</v>
@@ -858,7 +858,7 @@
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>-2.08</v>
+        <v>-2.14</v>
       </c>
       <c r="Q8" t="inlineStr"/>
     </row>
@@ -887,7 +887,7 @@
         <v>40.33</v>
       </c>
       <c r="H9" t="n">
-        <v>36.44</v>
+        <v>36.95</v>
       </c>
       <c r="I9" t="n">
         <v>10</v>
@@ -907,7 +907,7 @@
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>-0.97</v>
+        <v>-0.84</v>
       </c>
       <c r="Q9" t="inlineStr"/>
     </row>
@@ -936,7 +936,7 @@
         <v>127.16</v>
       </c>
       <c r="H10" t="n">
-        <v>139.38</v>
+        <v>137.42</v>
       </c>
       <c r="I10" t="n">
         <v>19.99</v>
@@ -956,7 +956,7 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>1.92</v>
+        <v>1.61</v>
       </c>
       <c r="Q10" t="inlineStr"/>
     </row>
@@ -985,7 +985,7 @@
         <v>196.9</v>
       </c>
       <c r="H11" t="n">
-        <v>197.55</v>
+        <v>196.05</v>
       </c>
       <c r="I11" t="n">
         <v>14.98</v>
@@ -1005,7 +1005,7 @@
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>0.05</v>
+        <v>-0.06</v>
       </c>
       <c r="Q11" t="inlineStr"/>
     </row>
@@ -1034,7 +1034,7 @@
         <v>33.66</v>
       </c>
       <c r="H12" t="n">
-        <v>32.31</v>
+        <v>31.46</v>
       </c>
       <c r="I12" t="n">
         <v>10</v>
@@ -1054,7 +1054,7 @@
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>-0.4</v>
+        <v>-0.66</v>
       </c>
       <c r="Q12" t="inlineStr"/>
     </row>
@@ -1083,7 +1083,7 @@
         <v>77.53</v>
       </c>
       <c r="H13" t="n">
-        <v>68.01000000000001</v>
+        <v>67.20999999999999</v>
       </c>
       <c r="I13" t="n">
         <v>14.99</v>
@@ -1103,7 +1103,7 @@
         <v>0</v>
       </c>
       <c r="P13" t="n">
-        <v>-1.84</v>
+        <v>-2</v>
       </c>
       <c r="Q13" t="inlineStr"/>
     </row>
@@ -1132,7 +1132,7 @@
         <v>160.64</v>
       </c>
       <c r="H14" t="n">
-        <v>172.84</v>
+        <v>172.3</v>
       </c>
       <c r="I14" t="n">
         <v>19.98</v>
@@ -1152,7 +1152,7 @@
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>1.52</v>
+        <v>1.45</v>
       </c>
       <c r="Q14" t="inlineStr"/>
     </row>
@@ -1181,7 +1181,7 @@
         <v>128.46</v>
       </c>
       <c r="H15" t="n">
-        <v>155.71</v>
+        <v>156.05</v>
       </c>
       <c r="I15" t="n">
         <v>11</v>
@@ -1201,7 +1201,7 @@
         <v>0</v>
       </c>
       <c r="P15" t="n">
-        <v>2.33</v>
+        <v>2.36</v>
       </c>
       <c r="Q15" t="inlineStr"/>
     </row>
@@ -1230,7 +1230,7 @@
         <v>20.62</v>
       </c>
       <c r="H16" t="n">
-        <v>17.3</v>
+        <v>17.17</v>
       </c>
       <c r="I16" t="n">
         <v>9.99</v>
@@ -1250,7 +1250,7 @@
         <v>0</v>
       </c>
       <c r="P16" t="n">
-        <v>-1.6</v>
+        <v>-1.67</v>
       </c>
       <c r="Q16" t="inlineStr"/>
     </row>
@@ -1279,7 +1279,7 @@
         <v>17.86</v>
       </c>
       <c r="H17" t="n">
-        <v>17.88</v>
+        <v>17.63</v>
       </c>
       <c r="I17" t="n">
         <v>17.86</v>
@@ -1299,7 +1299,7 @@
         <v>0</v>
       </c>
       <c r="P17" t="n">
-        <v>0.02</v>
+        <v>-0.23</v>
       </c>
       <c r="Q17" t="inlineStr"/>
     </row>
@@ -1328,7 +1328,7 @@
         <v>21.31</v>
       </c>
       <c r="H18" t="n">
-        <v>17.3</v>
+        <v>17.17</v>
       </c>
       <c r="I18" t="n">
         <v>20</v>
@@ -1348,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="P18" t="n">
-        <v>-3.76</v>
+        <v>-3.89</v>
       </c>
       <c r="Q18" t="inlineStr"/>
     </row>
@@ -1377,7 +1377,7 @@
         <v>232.2</v>
       </c>
       <c r="H19" t="n">
-        <v>200.14</v>
+        <v>200.41</v>
       </c>
       <c r="I19" t="n">
         <v>0.02</v>
@@ -1426,7 +1426,7 @@
         <v>56.78</v>
       </c>
       <c r="H20" t="n">
-        <v>59.59</v>
+        <v>59.48</v>
       </c>
       <c r="I20" t="n">
         <v>15</v>
@@ -1446,7 +1446,7 @@
         <v>0</v>
       </c>
       <c r="P20" t="n">
-        <v>0.74</v>
+        <v>0.71</v>
       </c>
       <c r="Q20" t="inlineStr"/>
     </row>
@@ -1475,7 +1475,7 @@
         <v>20.58</v>
       </c>
       <c r="H21" t="n">
-        <v>20.66</v>
+        <v>20.41</v>
       </c>
       <c r="I21" t="n">
         <v>20.58</v>
@@ -1495,7 +1495,7 @@
         <v>0</v>
       </c>
       <c r="P21" t="n">
-        <v>0.08</v>
+        <v>-0.17</v>
       </c>
       <c r="Q21" t="inlineStr"/>
     </row>
@@ -1524,7 +1524,7 @@
         <v>524.4299999999999</v>
       </c>
       <c r="H22" t="n">
-        <v>573.11</v>
+        <v>575.73</v>
       </c>
       <c r="I22" t="n">
         <v>0.52</v>
@@ -1544,7 +1544,7 @@
         <v>0</v>
       </c>
       <c r="P22" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="Q22" t="inlineStr"/>
     </row>
@@ -1573,7 +1573,7 @@
         <v>30.54</v>
       </c>
       <c r="H23" t="n">
-        <v>30.02</v>
+        <v>30.82</v>
       </c>
       <c r="I23" t="n">
         <v>10</v>
@@ -1593,7 +1593,7 @@
         <v>0</v>
       </c>
       <c r="P23" t="n">
-        <v>-0.17</v>
+        <v>0.09</v>
       </c>
       <c r="Q23" t="inlineStr"/>
     </row>
@@ -1622,7 +1622,7 @@
         <v>147.48</v>
       </c>
       <c r="H24" t="n">
-        <v>142.76</v>
+        <v>142.67</v>
       </c>
       <c r="I24" t="n">
         <v>3.41</v>
@@ -1671,7 +1671,7 @@
         <v>74.13</v>
       </c>
       <c r="H25" t="n">
-        <v>72.51000000000001</v>
+        <v>72.38</v>
       </c>
       <c r="I25" t="n">
         <v>74.13</v>
@@ -1691,7 +1691,7 @@
         <v>0</v>
       </c>
       <c r="P25" t="n">
-        <v>-1.62</v>
+        <v>-1.75</v>
       </c>
       <c r="Q25" t="inlineStr"/>
     </row>
@@ -1720,7 +1720,7 @@
         <v>38.23</v>
       </c>
       <c r="H26" t="n">
-        <v>32.31</v>
+        <v>31.46</v>
       </c>
       <c r="I26" t="n">
         <v>19.98</v>
@@ -1740,7 +1740,7 @@
         <v>0</v>
       </c>
       <c r="P26" t="n">
-        <v>-3.09</v>
+        <v>-3.54</v>
       </c>
       <c r="Q26" t="inlineStr"/>
     </row>
@@ -1769,7 +1769,7 @@
         <v>165.93</v>
       </c>
       <c r="H27" t="n">
-        <v>131.35</v>
+        <v>130.65</v>
       </c>
       <c r="I27" t="n">
         <v>17.94</v>
@@ -1789,7 +1789,7 @@
         <v>0</v>
       </c>
       <c r="P27" t="n">
-        <v>-3.73</v>
+        <v>-3.81</v>
       </c>
       <c r="Q27" t="inlineStr"/>
     </row>
@@ -1818,7 +1818,7 @@
         <v>27.17</v>
       </c>
       <c r="H28" t="n">
-        <v>36.44</v>
+        <v>36.95</v>
       </c>
       <c r="I28" t="n">
         <v>9.98</v>
@@ -1838,7 +1838,7 @@
         <v>0</v>
       </c>
       <c r="P28" t="n">
-        <v>3.4</v>
+        <v>3.59</v>
       </c>
       <c r="Q28" t="inlineStr"/>
     </row>
@@ -1867,7 +1867,7 @@
         <v>77.34999999999999</v>
       </c>
       <c r="H29" t="n">
-        <v>68.01000000000001</v>
+        <v>67.20999999999999</v>
       </c>
       <c r="I29" t="n">
         <v>19.99</v>
@@ -1887,7 +1887,7 @@
         <v>0</v>
       </c>
       <c r="P29" t="n">
-        <v>-2.41</v>
+        <v>-2.62</v>
       </c>
       <c r="Q29" t="inlineStr"/>
     </row>
@@ -1916,7 +1916,7 @@
         <v>129.17</v>
       </c>
       <c r="H30" t="n">
-        <v>131.35</v>
+        <v>130.65</v>
       </c>
       <c r="I30" t="n">
         <v>20</v>
@@ -1936,7 +1936,7 @@
         <v>0</v>
       </c>
       <c r="P30" t="n">
-        <v>0.33</v>
+        <v>0.22</v>
       </c>
       <c r="Q30" t="inlineStr"/>
     </row>
@@ -1965,7 +1965,7 @@
         <v>12.75</v>
       </c>
       <c r="H31" t="n">
-        <v>13.54</v>
+        <v>13.26</v>
       </c>
       <c r="I31" t="n">
         <v>14.49</v>
@@ -1985,7 +1985,7 @@
         <v>0</v>
       </c>
       <c r="P31" t="n">
-        <v>0.77</v>
+        <v>0.4</v>
       </c>
       <c r="Q31" t="inlineStr"/>
     </row>
@@ -2014,7 +2014,7 @@
         <v>24.11</v>
       </c>
       <c r="H32" t="n">
-        <v>17.3</v>
+        <v>17.17</v>
       </c>
       <c r="I32" t="n">
         <v>9.99</v>
@@ -2034,7 +2034,7 @@
         <v>0</v>
       </c>
       <c r="P32" t="n">
-        <v>-2.82</v>
+        <v>-2.87</v>
       </c>
       <c r="Q32" t="inlineStr"/>
     </row>
@@ -2063,7 +2063,7 @@
         <v>156.9</v>
       </c>
       <c r="H33" t="n">
-        <v>155.71</v>
+        <v>156.05</v>
       </c>
       <c r="I33" t="n">
         <v>15</v>
@@ -2083,7 +2083,7 @@
         <v>0</v>
       </c>
       <c r="P33" t="n">
-        <v>-0.11</v>
+        <v>-0.08</v>
       </c>
       <c r="Q33" t="inlineStr"/>
     </row>
@@ -2112,7 +2112,7 @@
         <v>52.83</v>
       </c>
       <c r="H34" t="n">
-        <v>59.59</v>
+        <v>59.48</v>
       </c>
       <c r="I34" t="n">
         <v>15</v>
@@ -2132,7 +2132,7 @@
         <v>0</v>
       </c>
       <c r="P34" t="n">
-        <v>1.92</v>
+        <v>1.89</v>
       </c>
       <c r="Q34" t="inlineStr"/>
     </row>
@@ -2161,7 +2161,7 @@
         <v>130.51</v>
       </c>
       <c r="H35" t="n">
-        <v>143.97</v>
+        <v>143.07</v>
       </c>
       <c r="I35" t="n">
         <v>0.04</v>
@@ -2188,11 +2188,11 @@
     <row r="36">
       <c r="A36" t="inlineStr"/>
       <c r="B36" t="n">
-        <v>1633116336</v>
+        <v>1845429980</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>VWO</t>
+          <t>BBVA.MC</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2204,16 +2204,16 @@
         <v>1</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>45686.83272234954</v>
+        <v>45805.66181400463</v>
       </c>
       <c r="G36" t="n">
-        <v>44.24</v>
+        <v>13.27</v>
       </c>
       <c r="H36" t="n">
-        <v>47.61</v>
+        <v>13.26</v>
       </c>
       <c r="I36" t="n">
-        <v>44.24</v>
+        <v>15.09</v>
       </c>
       <c r="J36" t="inlineStr"/>
       <c r="K36" t="inlineStr"/>
@@ -2230,18 +2230,18 @@
         <v>0</v>
       </c>
       <c r="P36" t="n">
-        <v>3.37</v>
+        <v>-0.2</v>
       </c>
       <c r="Q36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr"/>
       <c r="B37" t="n">
-        <v>1381375440</v>
+        <v>1633116336</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>VWO</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2250,19 +2250,19 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>0.1057</v>
+        <v>1</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>45484.67118315972</v>
+        <v>45686.83272234954</v>
       </c>
       <c r="G37" t="n">
-        <v>189.11</v>
+        <v>44.24</v>
       </c>
       <c r="H37" t="n">
-        <v>197.55</v>
+        <v>47.33</v>
       </c>
       <c r="I37" t="n">
-        <v>19.99</v>
+        <v>44.24</v>
       </c>
       <c r="J37" t="inlineStr"/>
       <c r="K37" t="inlineStr"/>
@@ -2279,18 +2279,18 @@
         <v>0</v>
       </c>
       <c r="P37" t="n">
-        <v>0.89</v>
+        <v>3.09</v>
       </c>
       <c r="Q37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr"/>
       <c r="B38" t="n">
-        <v>1806980482</v>
+        <v>1381375440</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>BCS</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2299,19 +2299,19 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>0.2406</v>
+        <v>0.1057</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>45783.83189613426</v>
+        <v>45484.67118315972</v>
       </c>
       <c r="G38" t="n">
-        <v>16.12</v>
+        <v>189.11</v>
       </c>
       <c r="H38" t="n">
-        <v>17.88</v>
+        <v>196.05</v>
       </c>
       <c r="I38" t="n">
-        <v>3.88</v>
+        <v>19.99</v>
       </c>
       <c r="J38" t="inlineStr"/>
       <c r="K38" t="inlineStr"/>
@@ -2328,18 +2328,18 @@
         <v>0</v>
       </c>
       <c r="P38" t="n">
-        <v>0.42</v>
+        <v>0.73</v>
       </c>
       <c r="Q38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr"/>
       <c r="B39" t="n">
-        <v>1680991980</v>
+        <v>1806980482</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>BCS</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2348,19 +2348,19 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>0.1958</v>
+        <v>0.2406</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>45716.8556621875</v>
+        <v>45783.83189613426</v>
       </c>
       <c r="G39" t="n">
-        <v>178.67</v>
+        <v>16.12</v>
       </c>
       <c r="H39" t="n">
-        <v>197.55</v>
+        <v>17.63</v>
       </c>
       <c r="I39" t="n">
-        <v>34.98</v>
+        <v>3.88</v>
       </c>
       <c r="J39" t="inlineStr"/>
       <c r="K39" t="inlineStr"/>
@@ -2377,18 +2377,18 @@
         <v>0</v>
       </c>
       <c r="P39" t="n">
-        <v>3.7</v>
+        <v>0.36</v>
       </c>
       <c r="Q39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr"/>
       <c r="B40" t="n">
-        <v>1843470413</v>
+        <v>1680991980</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CIB</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2397,19 +2397,19 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>0.4729</v>
+        <v>0.1958</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>45804.66637251157</v>
+        <v>45716.8556621875</v>
       </c>
       <c r="G40" t="n">
-        <v>42.29</v>
+        <v>178.67</v>
       </c>
       <c r="H40" t="n">
-        <v>42.18</v>
+        <v>196.05</v>
       </c>
       <c r="I40" t="n">
-        <v>20</v>
+        <v>34.98</v>
       </c>
       <c r="J40" t="inlineStr"/>
       <c r="K40" t="inlineStr"/>
@@ -2426,18 +2426,18 @@
         <v>0</v>
       </c>
       <c r="P40" t="n">
-        <v>-0.05</v>
+        <v>3.41</v>
       </c>
       <c r="Q40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr"/>
       <c r="B41" t="n">
-        <v>1662993636</v>
+        <v>1843470413</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>ACI</t>
+          <t>CIB</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2446,19 +2446,19 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>1</v>
+        <v>0.4729</v>
       </c>
       <c r="F41" s="2" t="n">
-        <v>45706.87026833333</v>
+        <v>45804.66637251157</v>
       </c>
       <c r="G41" t="n">
-        <v>20.65</v>
+        <v>42.29</v>
       </c>
       <c r="H41" t="n">
-        <v>22.18</v>
+        <v>42.16</v>
       </c>
       <c r="I41" t="n">
-        <v>20.65</v>
+        <v>20</v>
       </c>
       <c r="J41" t="inlineStr"/>
       <c r="K41" t="inlineStr"/>
@@ -2475,18 +2475,18 @@
         <v>0</v>
       </c>
       <c r="P41" t="n">
-        <v>1.53</v>
+        <v>-0.06</v>
       </c>
       <c r="Q41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr"/>
       <c r="B42" t="n">
-        <v>1481609355</v>
+        <v>1662993636</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>KMB</t>
+          <t>ACI</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2495,19 +2495,19 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>0.107</v>
+        <v>1</v>
       </c>
       <c r="F42" s="2" t="n">
-        <v>45568.7734872338</v>
+        <v>45706.87026833333</v>
       </c>
       <c r="G42" t="n">
-        <v>140.18</v>
+        <v>20.65</v>
       </c>
       <c r="H42" t="n">
-        <v>142.76</v>
+        <v>22.16</v>
       </c>
       <c r="I42" t="n">
-        <v>15</v>
+        <v>20.65</v>
       </c>
       <c r="J42" t="inlineStr"/>
       <c r="K42" t="inlineStr"/>
@@ -2524,18 +2524,18 @@
         <v>0</v>
       </c>
       <c r="P42" t="n">
-        <v>0.28</v>
+        <v>1.51</v>
       </c>
       <c r="Q42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr"/>
       <c r="B43" t="n">
-        <v>1744767540</v>
+        <v>1481609355</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>KMB</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2544,19 +2544,19 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>0.643</v>
+        <v>0.107</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>45751.72316712963</v>
+        <v>45568.7734872338</v>
       </c>
       <c r="G43" t="n">
-        <v>15.55</v>
+        <v>140.18</v>
       </c>
       <c r="H43" t="n">
-        <v>17.3</v>
+        <v>142.67</v>
       </c>
       <c r="I43" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J43" t="inlineStr"/>
       <c r="K43" t="inlineStr"/>
@@ -2573,18 +2573,18 @@
         <v>0</v>
       </c>
       <c r="P43" t="n">
-        <v>1.12</v>
+        <v>0.27</v>
       </c>
       <c r="Q43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr"/>
       <c r="B44" t="n">
-        <v>1817256440</v>
+        <v>1744767540</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2593,16 +2593,16 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>0.2267</v>
+        <v>0.643</v>
       </c>
       <c r="F44" s="2" t="n">
-        <v>45789.64787115741</v>
+        <v>45751.72316712963</v>
       </c>
       <c r="G44" t="n">
-        <v>44.1</v>
+        <v>15.55</v>
       </c>
       <c r="H44" t="n">
-        <v>43.88</v>
+        <v>17.17</v>
       </c>
       <c r="I44" t="n">
         <v>10</v>
@@ -2622,18 +2622,18 @@
         <v>0</v>
       </c>
       <c r="P44" t="n">
-        <v>-0.05</v>
+        <v>1.04</v>
       </c>
       <c r="Q44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr"/>
       <c r="B45" t="n">
-        <v>1843468958</v>
+        <v>1817256440</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2642,19 +2642,19 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>0.2208</v>
+        <v>0.2267</v>
       </c>
       <c r="F45" s="2" t="n">
-        <v>45804.66597149306</v>
+        <v>45789.64787115741</v>
       </c>
       <c r="G45" t="n">
-        <v>67.93000000000001</v>
+        <v>44.1</v>
       </c>
       <c r="H45" t="n">
-        <v>68.01000000000001</v>
+        <v>43.27</v>
       </c>
       <c r="I45" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J45" t="inlineStr"/>
       <c r="K45" t="inlineStr"/>
@@ -2671,18 +2671,18 @@
         <v>0</v>
       </c>
       <c r="P45" t="n">
-        <v>0.02</v>
+        <v>-0.19</v>
       </c>
       <c r="Q45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr"/>
       <c r="B46" t="n">
-        <v>1532661507</v>
+        <v>1843468958</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2691,19 +2691,19 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>0.06809999999999999</v>
+        <v>0.2208</v>
       </c>
       <c r="F46" s="2" t="n">
-        <v>45608.74251107639</v>
+        <v>45804.66597149306</v>
       </c>
       <c r="G46" t="n">
-        <v>190.67</v>
+        <v>67.93000000000001</v>
       </c>
       <c r="H46" t="n">
-        <v>197.55</v>
+        <v>67.20999999999999</v>
       </c>
       <c r="I46" t="n">
-        <v>12.98</v>
+        <v>15</v>
       </c>
       <c r="J46" t="inlineStr"/>
       <c r="K46" t="inlineStr"/>
@@ -2720,18 +2720,18 @@
         <v>0</v>
       </c>
       <c r="P46" t="n">
-        <v>0.47</v>
+        <v>-0.16</v>
       </c>
       <c r="Q46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr"/>
       <c r="B47" t="n">
-        <v>1583696868</v>
+        <v>1532661507</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>BOTZ.L</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2740,19 +2740,19 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>0.5</v>
+        <v>0.06809999999999999</v>
       </c>
       <c r="F47" s="2" t="n">
-        <v>45646.60053979167</v>
+        <v>45608.74251107639</v>
       </c>
       <c r="G47" t="n">
-        <v>20.645</v>
+        <v>190.67</v>
       </c>
       <c r="H47" t="n">
-        <v>20.66</v>
+        <v>196.05</v>
       </c>
       <c r="I47" t="n">
-        <v>10.32</v>
+        <v>12.98</v>
       </c>
       <c r="J47" t="inlineStr"/>
       <c r="K47" t="inlineStr"/>
@@ -2769,18 +2769,18 @@
         <v>0</v>
       </c>
       <c r="P47" t="n">
-        <v>0.01</v>
+        <v>0.37</v>
       </c>
       <c r="Q47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr"/>
       <c r="B48" t="n">
-        <v>1712849726</v>
+        <v>1583696868</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>FSLR</t>
+          <t>BOTZ.L</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2789,19 +2789,19 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>0.0861</v>
+        <v>0.5</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>45734.85489405093</v>
+        <v>45646.60053979167</v>
       </c>
       <c r="G48" t="n">
-        <v>127.72</v>
+        <v>20.645</v>
       </c>
       <c r="H48" t="n">
-        <v>155.71</v>
+        <v>20.41</v>
       </c>
       <c r="I48" t="n">
-        <v>11</v>
+        <v>10.32</v>
       </c>
       <c r="J48" t="inlineStr"/>
       <c r="K48" t="inlineStr"/>
@@ -2818,18 +2818,18 @@
         <v>0</v>
       </c>
       <c r="P48" t="n">
-        <v>2.41</v>
+        <v>-0.11</v>
       </c>
       <c r="Q48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr"/>
       <c r="B49" t="n">
-        <v>1582723120</v>
+        <v>1712849726</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>FSLR</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2838,19 +2838,19 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>0.3755</v>
+        <v>0.0861</v>
       </c>
       <c r="F49" s="2" t="n">
-        <v>45645.89511640046</v>
+        <v>45734.85489405093</v>
       </c>
       <c r="G49" t="n">
-        <v>53.26</v>
+        <v>127.72</v>
       </c>
       <c r="H49" t="n">
-        <v>59.59</v>
+        <v>156.05</v>
       </c>
       <c r="I49" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="J49" t="inlineStr"/>
       <c r="K49" t="inlineStr"/>
@@ -2867,18 +2867,18 @@
         <v>0</v>
       </c>
       <c r="P49" t="n">
-        <v>2.38</v>
+        <v>2.44</v>
       </c>
       <c r="Q49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr"/>
       <c r="B50" t="n">
-        <v>1806979127</v>
+        <v>1582723120</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2887,19 +2887,19 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>0.6361</v>
+        <v>0.3755</v>
       </c>
       <c r="F50" s="2" t="n">
-        <v>45783.83125244213</v>
+        <v>45645.89511640046</v>
       </c>
       <c r="G50" t="n">
-        <v>15.72</v>
+        <v>53.26</v>
       </c>
       <c r="H50" t="n">
-        <v>17.3</v>
+        <v>59.48</v>
       </c>
       <c r="I50" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="J50" t="inlineStr"/>
       <c r="K50" t="inlineStr"/>
@@ -2916,18 +2916,18 @@
         <v>0</v>
       </c>
       <c r="P50" t="n">
-        <v>1</v>
+        <v>2.33</v>
       </c>
       <c r="Q50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr"/>
       <c r="B51" t="n">
-        <v>1727591551</v>
+        <v>1806979127</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>BND</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2936,19 +2936,19 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>1</v>
+        <v>0.6361</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>45743.77389555555</v>
+        <v>45783.83125244213</v>
       </c>
       <c r="G51" t="n">
-        <v>72.87</v>
+        <v>15.72</v>
       </c>
       <c r="H51" t="n">
-        <v>72.51000000000001</v>
+        <v>17.17</v>
       </c>
       <c r="I51" t="n">
-        <v>72.87</v>
+        <v>10</v>
       </c>
       <c r="J51" t="inlineStr"/>
       <c r="K51" t="inlineStr"/>
@@ -2965,18 +2965,18 @@
         <v>0</v>
       </c>
       <c r="P51" t="n">
-        <v>-0.36</v>
+        <v>0.92</v>
       </c>
       <c r="Q51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr"/>
       <c r="B52" t="n">
-        <v>1666459270</v>
+        <v>1727591551</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ING</t>
+          <t>BND</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -2988,16 +2988,16 @@
         <v>1</v>
       </c>
       <c r="F52" s="2" t="n">
-        <v>45708.68166530092</v>
+        <v>45743.77389555555</v>
       </c>
       <c r="G52" t="n">
-        <v>17.18</v>
+        <v>72.87</v>
       </c>
       <c r="H52" t="n">
-        <v>21.3</v>
+        <v>72.38</v>
       </c>
       <c r="I52" t="n">
-        <v>17.18</v>
+        <v>72.87</v>
       </c>
       <c r="J52" t="inlineStr"/>
       <c r="K52" t="inlineStr"/>
@@ -3014,18 +3014,18 @@
         <v>0</v>
       </c>
       <c r="P52" t="n">
-        <v>4.12</v>
+        <v>-0.49</v>
       </c>
       <c r="Q52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr"/>
       <c r="B53" t="n">
-        <v>1648740228</v>
+        <v>1666459270</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>GOOGL</t>
+          <t>ING</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3034,19 +3034,19 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>0.0538</v>
+        <v>1</v>
       </c>
       <c r="F53" s="2" t="n">
-        <v>45695.85792408565</v>
+        <v>45708.68166530092</v>
       </c>
       <c r="G53" t="n">
-        <v>185.82</v>
+        <v>17.18</v>
       </c>
       <c r="H53" t="n">
-        <v>172.84</v>
+        <v>20.97</v>
       </c>
       <c r="I53" t="n">
-        <v>10</v>
+        <v>17.18</v>
       </c>
       <c r="J53" t="inlineStr"/>
       <c r="K53" t="inlineStr"/>
@@ -3063,18 +3063,18 @@
         <v>0</v>
       </c>
       <c r="P53" t="n">
-        <v>-0.7</v>
+        <v>3.79</v>
       </c>
       <c r="Q53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr"/>
       <c r="B54" t="n">
-        <v>1631475148</v>
+        <v>1648740228</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>YPF</t>
+          <t>GOOGL</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3083,16 +3083,16 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>0.2592</v>
+        <v>0.0538</v>
       </c>
       <c r="F54" s="2" t="n">
-        <v>45685.83625201389</v>
+        <v>45695.85792408565</v>
       </c>
       <c r="G54" t="n">
-        <v>38.58</v>
+        <v>185.82</v>
       </c>
       <c r="H54" t="n">
-        <v>36.44</v>
+        <v>172.3</v>
       </c>
       <c r="I54" t="n">
         <v>10</v>
@@ -3112,18 +3112,18 @@
         <v>0</v>
       </c>
       <c r="P54" t="n">
-        <v>-0.55</v>
+        <v>-0.73</v>
       </c>
       <c r="Q54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr"/>
       <c r="B55" t="n">
-        <v>1644796307</v>
+        <v>1631475148</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>ACI</t>
+          <t>YPF</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3132,19 +3132,19 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>1</v>
+        <v>0.2592</v>
       </c>
       <c r="F55" s="2" t="n">
-        <v>45693.85501710648</v>
+        <v>45685.83625201389</v>
       </c>
       <c r="G55" t="n">
-        <v>20.36</v>
+        <v>38.58</v>
       </c>
       <c r="H55" t="n">
-        <v>22.18</v>
+        <v>36.95</v>
       </c>
       <c r="I55" t="n">
-        <v>20.36</v>
+        <v>10</v>
       </c>
       <c r="J55" t="inlineStr"/>
       <c r="K55" t="inlineStr"/>
@@ -3161,18 +3161,18 @@
         <v>0</v>
       </c>
       <c r="P55" t="n">
-        <v>1.82</v>
+        <v>-0.42</v>
       </c>
       <c r="Q55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr"/>
       <c r="B56" t="n">
-        <v>1517510856</v>
+        <v>1644796307</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>ACI</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3181,19 +3181,19 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>0.0602</v>
+        <v>1</v>
       </c>
       <c r="F56" s="2" t="n">
-        <v>45597.61014849537</v>
+        <v>45693.85501710648</v>
       </c>
       <c r="G56" t="n">
-        <v>166.03</v>
+        <v>20.36</v>
       </c>
       <c r="H56" t="n">
-        <v>131.35</v>
+        <v>22.16</v>
       </c>
       <c r="I56" t="n">
-        <v>10</v>
+        <v>20.36</v>
       </c>
       <c r="J56" t="inlineStr"/>
       <c r="K56" t="inlineStr"/>
@@ -3210,18 +3210,18 @@
         <v>0</v>
       </c>
       <c r="P56" t="n">
-        <v>-2.09</v>
+        <v>1.8</v>
       </c>
       <c r="Q56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr"/>
       <c r="B57" t="n">
-        <v>1680993370</v>
+        <v>1517510856</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>VWO</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3230,19 +3230,19 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>1</v>
+        <v>0.0602</v>
       </c>
       <c r="F57" s="2" t="n">
-        <v>45716.85638861111</v>
+        <v>45597.61014849537</v>
       </c>
       <c r="G57" t="n">
-        <v>44.49</v>
+        <v>166.03</v>
       </c>
       <c r="H57" t="n">
-        <v>47.61</v>
+        <v>130.65</v>
       </c>
       <c r="I57" t="n">
-        <v>44.49</v>
+        <v>10</v>
       </c>
       <c r="J57" t="inlineStr"/>
       <c r="K57" t="inlineStr"/>
@@ -3259,18 +3259,18 @@
         <v>0</v>
       </c>
       <c r="P57" t="n">
-        <v>3.12</v>
+        <v>-2.13</v>
       </c>
       <c r="Q57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr"/>
       <c r="B58" t="n">
-        <v>1843474191</v>
+        <v>1680993370</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ING</t>
+          <t>VWO</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3279,19 +3279,19 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>0.9372</v>
+        <v>1</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>45804.66699503472</v>
+        <v>45716.85638861111</v>
       </c>
       <c r="G58" t="n">
-        <v>21.33</v>
+        <v>44.49</v>
       </c>
       <c r="H58" t="n">
-        <v>21.3</v>
+        <v>47.33</v>
       </c>
       <c r="I58" t="n">
-        <v>19.99</v>
+        <v>44.49</v>
       </c>
       <c r="J58" t="inlineStr"/>
       <c r="K58" t="inlineStr"/>
@@ -3308,18 +3308,18 @@
         <v>0</v>
       </c>
       <c r="P58" t="n">
-        <v>-0.03</v>
+        <v>2.84</v>
       </c>
       <c r="Q58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr"/>
       <c r="B59" t="n">
-        <v>1422773288</v>
+        <v>1843474191</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>ING</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3328,19 +3328,19 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>0.483</v>
+        <v>0.9372</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>45518.84428523148</v>
+        <v>45804.66699503472</v>
       </c>
       <c r="G59" t="n">
-        <v>51.24</v>
+        <v>21.33</v>
       </c>
       <c r="H59" t="n">
-        <v>59.59</v>
+        <v>20.97</v>
       </c>
       <c r="I59" t="n">
-        <v>24.75</v>
+        <v>19.99</v>
       </c>
       <c r="J59" t="inlineStr"/>
       <c r="K59" t="inlineStr"/>
@@ -3357,18 +3357,18 @@
         <v>0</v>
       </c>
       <c r="P59" t="n">
-        <v>4.03</v>
+        <v>-0.34</v>
       </c>
       <c r="Q59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr"/>
       <c r="B60" t="n">
-        <v>1744916452</v>
+        <v>1422773288</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>ING</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3377,19 +3377,19 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>0.4245</v>
+        <v>0.483</v>
       </c>
       <c r="F60" s="2" t="n">
-        <v>45751.74230173611</v>
+        <v>45518.84428523148</v>
       </c>
       <c r="G60" t="n">
-        <v>17.54</v>
+        <v>51.24</v>
       </c>
       <c r="H60" t="n">
-        <v>21.3</v>
+        <v>59.48</v>
       </c>
       <c r="I60" t="n">
-        <v>7.45</v>
+        <v>24.75</v>
       </c>
       <c r="J60" t="inlineStr"/>
       <c r="K60" t="inlineStr"/>
@@ -3406,18 +3406,18 @@
         <v>0</v>
       </c>
       <c r="P60" t="n">
-        <v>1.59</v>
+        <v>3.98</v>
       </c>
       <c r="Q60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr"/>
       <c r="B61" t="n">
-        <v>1824475555</v>
+        <v>1744916452</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ACI</t>
+          <t>ING</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -3426,19 +3426,19 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>1</v>
+        <v>0.4245</v>
       </c>
       <c r="F61" s="2" t="n">
-        <v>45792.64702015046</v>
+        <v>45751.74230173611</v>
       </c>
       <c r="G61" t="n">
-        <v>21.66</v>
+        <v>17.54</v>
       </c>
       <c r="H61" t="n">
-        <v>22.18</v>
+        <v>20.97</v>
       </c>
       <c r="I61" t="n">
-        <v>21.66</v>
+        <v>7.45</v>
       </c>
       <c r="J61" t="inlineStr"/>
       <c r="K61" t="inlineStr"/>
@@ -3455,18 +3455,18 @@
         <v>0</v>
       </c>
       <c r="P61" t="n">
-        <v>0.52</v>
+        <v>1.45</v>
       </c>
       <c r="Q61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr"/>
       <c r="B62" t="n">
-        <v>1806980496</v>
+        <v>1824475555</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>BCS</t>
+          <t>ACI</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3478,16 +3478,16 @@
         <v>1</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>45783.83190503472</v>
+        <v>45792.64702015046</v>
       </c>
       <c r="G62" t="n">
-        <v>16.12</v>
+        <v>21.66</v>
       </c>
       <c r="H62" t="n">
-        <v>17.88</v>
+        <v>22.16</v>
       </c>
       <c r="I62" t="n">
-        <v>16.12</v>
+        <v>21.66</v>
       </c>
       <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr"/>
@@ -3504,18 +3504,18 @@
         <v>0</v>
       </c>
       <c r="P62" t="n">
-        <v>1.76</v>
+        <v>0.5</v>
       </c>
       <c r="Q62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr"/>
       <c r="B63" t="n">
-        <v>1599435465</v>
+        <v>1806980496</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>BCS</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -3524,19 +3524,19 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>0.0289</v>
+        <v>1</v>
       </c>
       <c r="F63" s="2" t="n">
-        <v>45663.73115600694</v>
+        <v>45783.83190503472</v>
       </c>
       <c r="G63" t="n">
-        <v>517.7</v>
+        <v>16.12</v>
       </c>
       <c r="H63" t="n">
-        <v>573.11</v>
+        <v>17.63</v>
       </c>
       <c r="I63" t="n">
-        <v>14.96</v>
+        <v>16.12</v>
       </c>
       <c r="J63" t="inlineStr"/>
       <c r="K63" t="inlineStr"/>
@@ -3553,18 +3553,18 @@
         <v>0</v>
       </c>
       <c r="P63" t="n">
-        <v>1.6</v>
+        <v>1.51</v>
       </c>
       <c r="Q63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr"/>
       <c r="B64" t="n">
-        <v>1559803221</v>
+        <v>1599435465</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>MA</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3573,19 +3573,19 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>0.092</v>
+        <v>0.0289</v>
       </c>
       <c r="F64" s="2" t="n">
-        <v>45628.85951927083</v>
+        <v>45663.73115600694</v>
       </c>
       <c r="G64" t="n">
-        <v>162.85</v>
+        <v>517.7</v>
       </c>
       <c r="H64" t="n">
-        <v>131.35</v>
+        <v>575.73</v>
       </c>
       <c r="I64" t="n">
-        <v>14.98</v>
+        <v>14.96</v>
       </c>
       <c r="J64" t="inlineStr"/>
       <c r="K64" t="inlineStr"/>
@@ -3602,18 +3602,18 @@
         <v>0</v>
       </c>
       <c r="P64" t="n">
-        <v>-2.9</v>
+        <v>1.68</v>
       </c>
       <c r="Q64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr"/>
       <c r="B65" t="n">
-        <v>1666451221</v>
+        <v>1559803221</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3622,19 +3622,19 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>0.0001</v>
+        <v>0.092</v>
       </c>
       <c r="F65" s="2" t="n">
-        <v>45708.68022634259</v>
+        <v>45628.85951927083</v>
       </c>
       <c r="G65" t="n">
-        <v>43</v>
+        <v>162.85</v>
       </c>
       <c r="H65" t="n">
-        <v>43.88</v>
+        <v>130.65</v>
       </c>
       <c r="I65" t="n">
-        <v>0</v>
+        <v>14.98</v>
       </c>
       <c r="J65" t="inlineStr"/>
       <c r="K65" t="inlineStr"/>
@@ -3651,18 +3651,18 @@
         <v>0</v>
       </c>
       <c r="P65" t="n">
-        <v>0</v>
+        <v>-2.96</v>
       </c>
       <c r="Q65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr"/>
       <c r="B66" t="n">
-        <v>1701100481</v>
+        <v>1666451221</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -3671,19 +3671,19 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>0.0873</v>
+        <v>0.0001</v>
       </c>
       <c r="F66" s="2" t="n">
-        <v>45727.87214378472</v>
+        <v>45708.68022634259</v>
       </c>
       <c r="G66" t="n">
-        <v>171.67</v>
+        <v>43</v>
       </c>
       <c r="H66" t="n">
-        <v>197.55</v>
+        <v>43.27</v>
       </c>
       <c r="I66" t="n">
-        <v>14.99</v>
+        <v>0</v>
       </c>
       <c r="J66" t="inlineStr"/>
       <c r="K66" t="inlineStr"/>
@@ -3700,18 +3700,18 @@
         <v>0</v>
       </c>
       <c r="P66" t="n">
-        <v>2.26</v>
+        <v>0</v>
       </c>
       <c r="Q66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr"/>
       <c r="B67" t="n">
-        <v>1599455288</v>
+        <v>1701100481</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>YPF</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -3720,19 +3720,19 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>0.2195</v>
+        <v>0.0873</v>
       </c>
       <c r="F67" s="2" t="n">
-        <v>45663.73750263889</v>
+        <v>45727.87214378472</v>
       </c>
       <c r="G67" t="n">
-        <v>45.55</v>
+        <v>171.67</v>
       </c>
       <c r="H67" t="n">
-        <v>36.44</v>
+        <v>196.05</v>
       </c>
       <c r="I67" t="n">
-        <v>10</v>
+        <v>14.99</v>
       </c>
       <c r="J67" t="inlineStr"/>
       <c r="K67" t="inlineStr"/>
@@ -3749,18 +3749,18 @@
         <v>0</v>
       </c>
       <c r="P67" t="n">
-        <v>-2</v>
+        <v>2.13</v>
       </c>
       <c r="Q67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr"/>
       <c r="B68" t="n">
-        <v>1811475599</v>
+        <v>1599455288</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>BBVA.MC</t>
+          <t>YPF</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3769,19 +3769,19 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>0.7256</v>
+        <v>0.2195</v>
       </c>
       <c r="F68" s="2" t="n">
-        <v>45785.66972070602</v>
+        <v>45663.73750263889</v>
       </c>
       <c r="G68" t="n">
-        <v>12.75</v>
+        <v>45.55</v>
       </c>
       <c r="H68" t="n">
-        <v>13.54</v>
+        <v>36.95</v>
       </c>
       <c r="I68" t="n">
-        <v>10.51</v>
+        <v>10</v>
       </c>
       <c r="J68" t="inlineStr"/>
       <c r="K68" t="inlineStr"/>
@@ -3798,18 +3798,18 @@
         <v>0</v>
       </c>
       <c r="P68" t="n">
-        <v>0.5600000000000001</v>
+        <v>-1.89</v>
       </c>
       <c r="Q68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr"/>
       <c r="B69" t="n">
-        <v>1727563010</v>
+        <v>1811475599</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>VWO</t>
+          <t>BBVA.MC</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3818,19 +3818,19 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>1</v>
+        <v>0.7256</v>
       </c>
       <c r="F69" s="2" t="n">
-        <v>45743.76106726852</v>
+        <v>45785.66972070602</v>
       </c>
       <c r="G69" t="n">
-        <v>46.11</v>
+        <v>12.75</v>
       </c>
       <c r="H69" t="n">
-        <v>47.61</v>
+        <v>13.26</v>
       </c>
       <c r="I69" t="n">
-        <v>46.11</v>
+        <v>10.51</v>
       </c>
       <c r="J69" t="inlineStr"/>
       <c r="K69" t="inlineStr"/>
@@ -3847,18 +3847,18 @@
         <v>0</v>
       </c>
       <c r="P69" t="n">
-        <v>1.5</v>
+        <v>0.3</v>
       </c>
       <c r="Q69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr"/>
       <c r="B70" t="n">
-        <v>1644789287</v>
+        <v>1727563010</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>KMB</t>
+          <t>VWO</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -3867,19 +3867,19 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>0.0813</v>
+        <v>1</v>
       </c>
       <c r="F70" s="2" t="n">
-        <v>45693.85123056713</v>
+        <v>45743.76106726852</v>
       </c>
       <c r="G70" t="n">
-        <v>129.08</v>
+        <v>46.11</v>
       </c>
       <c r="H70" t="n">
-        <v>142.76</v>
+        <v>47.33</v>
       </c>
       <c r="I70" t="n">
-        <v>10.49</v>
+        <v>46.11</v>
       </c>
       <c r="J70" t="inlineStr"/>
       <c r="K70" t="inlineStr"/>
@@ -3896,18 +3896,18 @@
         <v>0</v>
       </c>
       <c r="P70" t="n">
-        <v>1.12</v>
+        <v>1.22</v>
       </c>
       <c r="Q70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr"/>
       <c r="B71" t="n">
-        <v>1621495187</v>
+        <v>1644789287</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>YPF</t>
+          <t>KMB</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -3916,19 +3916,19 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>0.2318</v>
+        <v>0.0813</v>
       </c>
       <c r="F71" s="2" t="n">
-        <v>45678.83178196759</v>
+        <v>45693.85123056713</v>
       </c>
       <c r="G71" t="n">
-        <v>43.27</v>
+        <v>129.08</v>
       </c>
       <c r="H71" t="n">
-        <v>36.44</v>
+        <v>142.67</v>
       </c>
       <c r="I71" t="n">
-        <v>10.03</v>
+        <v>10.49</v>
       </c>
       <c r="J71" t="inlineStr"/>
       <c r="K71" t="inlineStr"/>
@@ -3945,18 +3945,18 @@
         <v>0</v>
       </c>
       <c r="P71" t="n">
-        <v>-1.58</v>
+        <v>1.11</v>
       </c>
       <c r="Q71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr"/>
       <c r="B72" t="n">
-        <v>1644788775</v>
+        <v>1621495187</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>YPF</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -3965,19 +3965,19 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>0.07580000000000001</v>
+        <v>0.2318</v>
       </c>
       <c r="F72" s="2" t="n">
-        <v>45693.85093391204</v>
+        <v>45678.83178196759</v>
       </c>
       <c r="G72" t="n">
-        <v>144.94</v>
+        <v>43.27</v>
       </c>
       <c r="H72" t="n">
-        <v>131.35</v>
+        <v>36.95</v>
       </c>
       <c r="I72" t="n">
-        <v>10.99</v>
+        <v>10.03</v>
       </c>
       <c r="J72" t="inlineStr"/>
       <c r="K72" t="inlineStr"/>
@@ -3994,18 +3994,18 @@
         <v>0</v>
       </c>
       <c r="P72" t="n">
-        <v>-1.03</v>
+        <v>-1.46</v>
       </c>
       <c r="Q72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr"/>
       <c r="B73" t="n">
-        <v>1495551484</v>
+        <v>1644788775</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>INGR</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -4014,19 +4014,19 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>0.1914</v>
+        <v>0.07580000000000001</v>
       </c>
       <c r="F73" s="2" t="n">
-        <v>45580.70648087963</v>
+        <v>45693.85093391204</v>
       </c>
       <c r="G73" t="n">
-        <v>135.82</v>
+        <v>144.94</v>
       </c>
       <c r="H73" t="n">
-        <v>139.38</v>
+        <v>130.65</v>
       </c>
       <c r="I73" t="n">
-        <v>26</v>
+        <v>10.99</v>
       </c>
       <c r="J73" t="inlineStr"/>
       <c r="K73" t="inlineStr"/>
@@ -4043,18 +4043,18 @@
         <v>0</v>
       </c>
       <c r="P73" t="n">
-        <v>0.68</v>
+        <v>-1.09</v>
       </c>
       <c r="Q73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr"/>
       <c r="B74" t="n">
-        <v>1830408508</v>
+        <v>1495551484</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>INGR</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -4063,19 +4063,19 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>0.5793</v>
+        <v>0.1914</v>
       </c>
       <c r="F74" s="2" t="n">
-        <v>45796.82346997685</v>
+        <v>45580.70648087963</v>
       </c>
       <c r="G74" t="n">
-        <v>17.26</v>
+        <v>135.82</v>
       </c>
       <c r="H74" t="n">
-        <v>17.3</v>
+        <v>137.42</v>
       </c>
       <c r="I74" t="n">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="J74" t="inlineStr"/>
       <c r="K74" t="inlineStr"/>
@@ -4092,18 +4092,18 @@
         <v>0</v>
       </c>
       <c r="P74" t="n">
-        <v>0.02</v>
+        <v>0.3</v>
       </c>
       <c r="Q74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr"/>
       <c r="B75" t="n">
-        <v>1563288050</v>
+        <v>1830408508</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -4112,16 +4112,16 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>0.0626</v>
+        <v>0.5793</v>
       </c>
       <c r="F75" s="2" t="n">
-        <v>45630.85583428241</v>
+        <v>45796.82346997685</v>
       </c>
       <c r="G75" t="n">
-        <v>159.74</v>
+        <v>17.26</v>
       </c>
       <c r="H75" t="n">
-        <v>131.35</v>
+        <v>17.17</v>
       </c>
       <c r="I75" t="n">
         <v>10</v>
@@ -4141,18 +4141,18 @@
         <v>0</v>
       </c>
       <c r="P75" t="n">
-        <v>-1.78</v>
+        <v>-0.05</v>
       </c>
       <c r="Q75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr"/>
       <c r="B76" t="n">
-        <v>1701100027</v>
+        <v>1563288050</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -4161,19 +4161,19 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>0.7812</v>
+        <v>0.0626</v>
       </c>
       <c r="F76" s="2" t="n">
-        <v>45727.87202070602</v>
+        <v>45630.85583428241</v>
       </c>
       <c r="G76" t="n">
-        <v>19.2</v>
+        <v>159.74</v>
       </c>
       <c r="H76" t="n">
-        <v>17.3</v>
+        <v>130.65</v>
       </c>
       <c r="I76" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="J76" t="inlineStr"/>
       <c r="K76" t="inlineStr"/>
@@ -4190,18 +4190,18 @@
         <v>0</v>
       </c>
       <c r="P76" t="n">
-        <v>-1.49</v>
+        <v>-1.82</v>
       </c>
       <c r="Q76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr"/>
       <c r="B77" t="n">
-        <v>1744929368</v>
+        <v>1845429956</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>BBVA.MC</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -4210,19 +4210,19 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>0.0192</v>
+        <v>0.6565</v>
       </c>
       <c r="F77" s="2" t="n">
-        <v>45751.74500871528</v>
+        <v>45805.66180811343</v>
       </c>
       <c r="G77" t="n">
-        <v>324.48</v>
+        <v>13.275</v>
       </c>
       <c r="H77" t="n">
-        <v>358.47</v>
+        <v>13.26</v>
       </c>
       <c r="I77" t="n">
-        <v>6.23</v>
+        <v>9.91</v>
       </c>
       <c r="J77" t="inlineStr"/>
       <c r="K77" t="inlineStr"/>
@@ -4239,18 +4239,18 @@
         <v>0</v>
       </c>
       <c r="P77" t="n">
-        <v>0.65</v>
+        <v>-0.13</v>
       </c>
       <c r="Q77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr"/>
       <c r="B78" t="n">
-        <v>1599431096</v>
+        <v>1701100027</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -4259,19 +4259,19 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>0.1013</v>
+        <v>0.7812</v>
       </c>
       <c r="F78" s="2" t="n">
-        <v>45663.73014731482</v>
+        <v>45727.87202070602</v>
       </c>
       <c r="G78" t="n">
-        <v>148.02</v>
+        <v>19.2</v>
       </c>
       <c r="H78" t="n">
-        <v>131.35</v>
+        <v>17.17</v>
       </c>
       <c r="I78" t="n">
-        <v>14.99</v>
+        <v>15</v>
       </c>
       <c r="J78" t="inlineStr"/>
       <c r="K78" t="inlineStr"/>
@@ -4288,18 +4288,18 @@
         <v>0</v>
       </c>
       <c r="P78" t="n">
-        <v>-1.68</v>
+        <v>-1.59</v>
       </c>
       <c r="Q78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr"/>
       <c r="B79" t="n">
-        <v>1554742887</v>
+        <v>1744929368</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>V</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -4308,19 +4308,19 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>0.08400000000000001</v>
+        <v>0.0192</v>
       </c>
       <c r="F79" s="2" t="n">
-        <v>45623.74993112269</v>
+        <v>45751.74500871528</v>
       </c>
       <c r="G79" t="n">
-        <v>178.48</v>
+        <v>324.48</v>
       </c>
       <c r="H79" t="n">
-        <v>197.55</v>
+        <v>359.84</v>
       </c>
       <c r="I79" t="n">
-        <v>14.99</v>
+        <v>6.23</v>
       </c>
       <c r="J79" t="inlineStr"/>
       <c r="K79" t="inlineStr"/>
@@ -4337,18 +4337,18 @@
         <v>0</v>
       </c>
       <c r="P79" t="n">
-        <v>1.6</v>
+        <v>0.68</v>
       </c>
       <c r="Q79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr"/>
       <c r="B80" t="n">
-        <v>1666459175</v>
+        <v>1599431096</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>ING</t>
+          <t>PEP</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -4357,19 +4357,19 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>0.1641</v>
+        <v>0.1013</v>
       </c>
       <c r="F80" s="2" t="n">
-        <v>45708.68165298611</v>
+        <v>45663.73014731482</v>
       </c>
       <c r="G80" t="n">
-        <v>17.18</v>
+        <v>148.02</v>
       </c>
       <c r="H80" t="n">
-        <v>21.3</v>
+        <v>130.65</v>
       </c>
       <c r="I80" t="n">
-        <v>2.82</v>
+        <v>14.99</v>
       </c>
       <c r="J80" t="inlineStr"/>
       <c r="K80" t="inlineStr"/>
@@ -4386,18 +4386,18 @@
         <v>0</v>
       </c>
       <c r="P80" t="n">
-        <v>0.68</v>
+        <v>-1.76</v>
       </c>
       <c r="Q80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr"/>
       <c r="B81" t="n">
-        <v>1824477589</v>
+        <v>1554742887</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -4406,19 +4406,19 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>0.2344</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="F81" s="2" t="n">
-        <v>45792.64732982639</v>
+        <v>45623.74993112269</v>
       </c>
       <c r="G81" t="n">
-        <v>42.66</v>
+        <v>178.48</v>
       </c>
       <c r="H81" t="n">
-        <v>43.88</v>
+        <v>196.05</v>
       </c>
       <c r="I81" t="n">
-        <v>10</v>
+        <v>14.99</v>
       </c>
       <c r="J81" t="inlineStr"/>
       <c r="K81" t="inlineStr"/>
@@ -4435,18 +4435,18 @@
         <v>0</v>
       </c>
       <c r="P81" t="n">
-        <v>0.29</v>
+        <v>1.48</v>
       </c>
       <c r="Q81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr"/>
       <c r="B82" t="n">
-        <v>1381417257</v>
+        <v>1666459175</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>BATT.AS</t>
+          <t>ING</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4455,19 +4455,19 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>1</v>
+        <v>0.1641</v>
       </c>
       <c r="F82" s="2" t="n">
-        <v>45484.67877329861</v>
+        <v>45708.68165298611</v>
       </c>
       <c r="G82" t="n">
-        <v>16.374</v>
+        <v>17.18</v>
       </c>
       <c r="H82" t="n">
-        <v>15.394</v>
+        <v>20.97</v>
       </c>
       <c r="I82" t="n">
-        <v>17.9</v>
+        <v>2.82</v>
       </c>
       <c r="J82" t="inlineStr"/>
       <c r="K82" t="inlineStr"/>
@@ -4484,18 +4484,18 @@
         <v>0</v>
       </c>
       <c r="P82" t="n">
-        <v>-0.55</v>
+        <v>0.62</v>
       </c>
       <c r="Q82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr"/>
       <c r="B83" t="n">
-        <v>1806977521</v>
+        <v>1824477589</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>YPF</t>
+          <t>EXC</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -4504,16 +4504,16 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>0.3367</v>
+        <v>0.2344</v>
       </c>
       <c r="F83" s="2" t="n">
-        <v>45783.8305750463</v>
+        <v>45792.64732982639</v>
       </c>
       <c r="G83" t="n">
-        <v>29.7</v>
+        <v>42.66</v>
       </c>
       <c r="H83" t="n">
-        <v>36.44</v>
+        <v>43.27</v>
       </c>
       <c r="I83" t="n">
         <v>10</v>
@@ -4533,18 +4533,18 @@
         <v>0</v>
       </c>
       <c r="P83" t="n">
-        <v>2.27</v>
+        <v>0.14</v>
       </c>
       <c r="Q83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr"/>
       <c r="B84" t="n">
-        <v>1727574394</v>
+        <v>1381417257</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>ACI</t>
+          <t>BATT.AS</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -4556,16 +4556,16 @@
         <v>1</v>
       </c>
       <c r="F84" s="2" t="n">
-        <v>45743.76658678241</v>
+        <v>45484.67877329861</v>
       </c>
       <c r="G84" t="n">
-        <v>21.13</v>
+        <v>16.374</v>
       </c>
       <c r="H84" t="n">
-        <v>22.18</v>
+        <v>15.382</v>
       </c>
       <c r="I84" t="n">
-        <v>21.13</v>
+        <v>17.9</v>
       </c>
       <c r="J84" t="inlineStr"/>
       <c r="K84" t="inlineStr"/>
@@ -4582,18 +4582,18 @@
         <v>0</v>
       </c>
       <c r="P84" t="n">
-        <v>1.05</v>
+        <v>-0.62</v>
       </c>
       <c r="Q84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr"/>
       <c r="B85" t="n">
-        <v>1461331124</v>
+        <v>1806977521</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>MO</t>
+          <t>YPF</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -4602,19 +4602,19 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>0.3922</v>
+        <v>0.3367</v>
       </c>
       <c r="F85" s="2" t="n">
-        <v>45553.65374138889</v>
+        <v>45783.8305750463</v>
       </c>
       <c r="G85" t="n">
-        <v>50.99</v>
+        <v>29.7</v>
       </c>
       <c r="H85" t="n">
-        <v>59.59</v>
+        <v>36.95</v>
       </c>
       <c r="I85" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="J85" t="inlineStr"/>
       <c r="K85" t="inlineStr"/>
@@ -4631,18 +4631,18 @@
         <v>0</v>
       </c>
       <c r="P85" t="n">
-        <v>3.37</v>
+        <v>2.44</v>
       </c>
       <c r="Q85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr"/>
       <c r="B86" t="n">
-        <v>1744879358</v>
+        <v>1727574394</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>ACI</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -4651,19 +4651,19 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>0.2701</v>
+        <v>1</v>
       </c>
       <c r="F86" s="2" t="n">
-        <v>45751.73925940973</v>
+        <v>45743.76658678241</v>
       </c>
       <c r="G86" t="n">
-        <v>148.09</v>
+        <v>21.13</v>
       </c>
       <c r="H86" t="n">
-        <v>197.55</v>
+        <v>22.16</v>
       </c>
       <c r="I86" t="n">
-        <v>40</v>
+        <v>21.13</v>
       </c>
       <c r="J86" t="inlineStr"/>
       <c r="K86" t="inlineStr"/>
@@ -4680,18 +4680,18 @@
         <v>0</v>
       </c>
       <c r="P86" t="n">
-        <v>13.36</v>
+        <v>1.03</v>
       </c>
       <c r="Q86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr"/>
       <c r="B87" t="n">
-        <v>1662995258</v>
+        <v>1461331124</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>NEE</t>
+          <t>MO</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -4700,16 +4700,16 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>0.2943</v>
+        <v>0.3922</v>
       </c>
       <c r="F87" s="2" t="n">
-        <v>45706.87121422453</v>
+        <v>45553.65374138889</v>
       </c>
       <c r="G87" t="n">
-        <v>67.97</v>
+        <v>50.99</v>
       </c>
       <c r="H87" t="n">
-        <v>68.01000000000001</v>
+        <v>59.48</v>
       </c>
       <c r="I87" t="n">
         <v>20</v>
@@ -4729,18 +4729,18 @@
         <v>0</v>
       </c>
       <c r="P87" t="n">
-        <v>0.02</v>
+        <v>3.33</v>
       </c>
       <c r="Q87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr"/>
       <c r="B88" t="n">
-        <v>1817264187</v>
+        <v>1744879358</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>CIB</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -4749,19 +4749,19 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>0.4757</v>
+        <v>0.2701</v>
       </c>
       <c r="F88" s="2" t="n">
-        <v>45789.64859377315</v>
+        <v>45751.73925940973</v>
       </c>
       <c r="G88" t="n">
-        <v>42.02</v>
+        <v>148.09</v>
       </c>
       <c r="H88" t="n">
-        <v>42.18</v>
+        <v>196.05</v>
       </c>
       <c r="I88" t="n">
-        <v>19.99</v>
+        <v>40</v>
       </c>
       <c r="J88" t="inlineStr"/>
       <c r="K88" t="inlineStr"/>
@@ -4778,18 +4778,18 @@
         <v>0</v>
       </c>
       <c r="P88" t="n">
-        <v>0.08</v>
+        <v>12.95</v>
       </c>
       <c r="Q88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr"/>
       <c r="B89" t="n">
-        <v>1754304266</v>
+        <v>1662995258</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>NEE</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -4798,19 +4798,19 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>0.7137</v>
+        <v>0.2943</v>
       </c>
       <c r="F89" s="2" t="n">
-        <v>45755.88055112268</v>
+        <v>45706.87121422453</v>
       </c>
       <c r="G89" t="n">
-        <v>14</v>
+        <v>67.97</v>
       </c>
       <c r="H89" t="n">
-        <v>17.3</v>
+        <v>67.20999999999999</v>
       </c>
       <c r="I89" t="n">
-        <v>9.99</v>
+        <v>20</v>
       </c>
       <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr"/>
@@ -4827,18 +4827,18 @@
         <v>0</v>
       </c>
       <c r="P89" t="n">
-        <v>2.36</v>
+        <v>-0.22</v>
       </c>
       <c r="Q89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr"/>
       <c r="B90" t="n">
-        <v>1554741956</v>
+        <v>1817264187</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>ING</t>
+          <t>CIB</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -4847,19 +4847,19 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>1</v>
+        <v>0.4757</v>
       </c>
       <c r="F90" s="2" t="n">
-        <v>45623.74952237269</v>
+        <v>45789.64859377315</v>
       </c>
       <c r="G90" t="n">
-        <v>15.3</v>
+        <v>42.02</v>
       </c>
       <c r="H90" t="n">
-        <v>21.3</v>
+        <v>42.16</v>
       </c>
       <c r="I90" t="n">
-        <v>15.3</v>
+        <v>19.99</v>
       </c>
       <c r="J90" t="inlineStr"/>
       <c r="K90" t="inlineStr"/>
@@ -4876,18 +4876,18 @@
         <v>0</v>
       </c>
       <c r="P90" t="n">
-        <v>6</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="Q90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr"/>
       <c r="B91" t="n">
-        <v>1701098878</v>
+        <v>1754304266</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>FSLR</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -4896,19 +4896,19 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>0.0383</v>
+        <v>0.7137</v>
       </c>
       <c r="F91" s="2" t="n">
-        <v>45727.87167594907</v>
+        <v>45755.88055112268</v>
       </c>
       <c r="G91" t="n">
-        <v>139.41</v>
+        <v>14</v>
       </c>
       <c r="H91" t="n">
-        <v>155.71</v>
+        <v>17.17</v>
       </c>
       <c r="I91" t="n">
-        <v>5.34</v>
+        <v>9.99</v>
       </c>
       <c r="J91" t="inlineStr"/>
       <c r="K91" t="inlineStr"/>
@@ -4925,18 +4925,18 @@
         <v>0</v>
       </c>
       <c r="P91" t="n">
-        <v>0.62</v>
+        <v>2.26</v>
       </c>
       <c r="Q91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr"/>
       <c r="B92" t="n">
-        <v>1806978791</v>
+        <v>1554741956</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>FSLR</t>
+          <t>ING</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -4945,19 +4945,19 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>0.0867</v>
+        <v>1</v>
       </c>
       <c r="F92" s="2" t="n">
-        <v>45783.83109655092</v>
+        <v>45623.74952237269</v>
       </c>
       <c r="G92" t="n">
-        <v>126.78</v>
+        <v>15.3</v>
       </c>
       <c r="H92" t="n">
-        <v>155.71</v>
+        <v>20.97</v>
       </c>
       <c r="I92" t="n">
-        <v>10.99</v>
+        <v>15.3</v>
       </c>
       <c r="J92" t="inlineStr"/>
       <c r="K92" t="inlineStr"/>
@@ -4974,18 +4974,18 @@
         <v>0</v>
       </c>
       <c r="P92" t="n">
-        <v>2.51</v>
+        <v>5.67</v>
       </c>
       <c r="Q92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr"/>
       <c r="B93" t="n">
-        <v>1582708979</v>
+        <v>1701098878</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>TSM</t>
+          <t>FSLR</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -4994,19 +4994,19 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>0.0769</v>
+        <v>0.0383</v>
       </c>
       <c r="F93" s="2" t="n">
-        <v>45645.88746980324</v>
+        <v>45727.87167594907</v>
       </c>
       <c r="G93" t="n">
-        <v>195.11</v>
+        <v>139.41</v>
       </c>
       <c r="H93" t="n">
-        <v>197.55</v>
+        <v>156.05</v>
       </c>
       <c r="I93" t="n">
-        <v>15</v>
+        <v>5.34</v>
       </c>
       <c r="J93" t="inlineStr"/>
       <c r="K93" t="inlineStr"/>
@@ -5023,18 +5023,18 @@
         <v>0</v>
       </c>
       <c r="P93" t="n">
-        <v>0.19</v>
+        <v>0.64</v>
       </c>
       <c r="Q93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr"/>
       <c r="B94" t="n">
-        <v>1559803984</v>
+        <v>1806978791</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>KMB</t>
+          <t>FSLR</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -5043,19 +5043,19 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>0.1076</v>
+        <v>0.0867</v>
       </c>
       <c r="F94" s="2" t="n">
-        <v>45628.86014383102</v>
+        <v>45783.83109655092</v>
       </c>
       <c r="G94" t="n">
-        <v>139.4</v>
+        <v>126.78</v>
       </c>
       <c r="H94" t="n">
-        <v>142.76</v>
+        <v>156.05</v>
       </c>
       <c r="I94" t="n">
-        <v>15</v>
+        <v>10.99</v>
       </c>
       <c r="J94" t="inlineStr"/>
       <c r="K94" t="inlineStr"/>
@@ -5072,18 +5072,18 @@
         <v>0</v>
       </c>
       <c r="P94" t="n">
-        <v>0.36</v>
+        <v>2.54</v>
       </c>
       <c r="Q94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr"/>
       <c r="B95" t="n">
-        <v>1666461140</v>
+        <v>1582708979</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>YPF</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -5092,19 +5092,19 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>0.2651</v>
+        <v>0.0769</v>
       </c>
       <c r="F95" s="2" t="n">
-        <v>45708.68207092593</v>
+        <v>45645.88746980324</v>
       </c>
       <c r="G95" t="n">
-        <v>37.7</v>
+        <v>195.11</v>
       </c>
       <c r="H95" t="n">
-        <v>36.44</v>
+        <v>196.05</v>
       </c>
       <c r="I95" t="n">
-        <v>9.99</v>
+        <v>15</v>
       </c>
       <c r="J95" t="inlineStr"/>
       <c r="K95" t="inlineStr"/>
@@ -5121,18 +5121,18 @@
         <v>0</v>
       </c>
       <c r="P95" t="n">
-        <v>-0.33</v>
+        <v>0.08</v>
       </c>
       <c r="Q95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr"/>
       <c r="B96" t="n">
-        <v>1635194724</v>
+        <v>1559803984</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>AGIO</t>
+          <t>KMB</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -5141,19 +5141,19 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>0.2875</v>
+        <v>0.1076</v>
       </c>
       <c r="F96" s="2" t="n">
-        <v>45687.85271734954</v>
+        <v>45628.86014383102</v>
       </c>
       <c r="G96" t="n">
-        <v>34.78</v>
+        <v>139.4</v>
       </c>
       <c r="H96" t="n">
-        <v>30.02</v>
+        <v>142.67</v>
       </c>
       <c r="I96" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="J96" t="inlineStr"/>
       <c r="K96" t="inlineStr"/>
@@ -5170,18 +5170,18 @@
         <v>0</v>
       </c>
       <c r="P96" t="n">
-        <v>-1.37</v>
+        <v>0.35</v>
       </c>
       <c r="Q96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr"/>
       <c r="B97" t="n">
-        <v>1648737122</v>
+        <v>1666461140</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>YPF</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -5190,19 +5190,19 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>0.0269</v>
+        <v>0.2651</v>
       </c>
       <c r="F97" s="2" t="n">
-        <v>45695.85619950231</v>
+        <v>45708.68207092593</v>
       </c>
       <c r="G97" t="n">
-        <v>408.33</v>
+        <v>37.7</v>
       </c>
       <c r="H97" t="n">
-        <v>460.45</v>
+        <v>36.95</v>
       </c>
       <c r="I97" t="n">
-        <v>10.98</v>
+        <v>9.99</v>
       </c>
       <c r="J97" t="inlineStr"/>
       <c r="K97" t="inlineStr"/>
@@ -5219,18 +5219,18 @@
         <v>0</v>
       </c>
       <c r="P97" t="n">
-        <v>1.41</v>
+        <v>-0.19</v>
       </c>
       <c r="Q97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr"/>
       <c r="B98" t="n">
-        <v>1648733962</v>
+        <v>1635194724</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>KMB</t>
+          <t>AGIO</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -5239,19 +5239,19 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>0.081</v>
+        <v>0.2875</v>
       </c>
       <c r="F98" s="2" t="n">
-        <v>45695.85463682871</v>
+        <v>45687.85271734954</v>
       </c>
       <c r="G98" t="n">
-        <v>129.56</v>
+        <v>34.78</v>
       </c>
       <c r="H98" t="n">
-        <v>142.76</v>
+        <v>30.82</v>
       </c>
       <c r="I98" t="n">
-        <v>10.49</v>
+        <v>10</v>
       </c>
       <c r="J98" t="inlineStr"/>
       <c r="K98" t="inlineStr"/>
@@ -5268,18 +5268,18 @@
         <v>0</v>
       </c>
       <c r="P98" t="n">
-        <v>1.07</v>
+        <v>-1.14</v>
       </c>
       <c r="Q98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr"/>
       <c r="B99" t="n">
-        <v>1680994777</v>
+        <v>1648737122</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -5288,19 +5288,19 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>0.7278</v>
+        <v>0.0269</v>
       </c>
       <c r="F99" s="2" t="n">
-        <v>45716.85705375</v>
+        <v>45695.85619950231</v>
       </c>
       <c r="G99" t="n">
-        <v>20.6</v>
+        <v>408.33</v>
       </c>
       <c r="H99" t="n">
-        <v>17.3</v>
+        <v>457.4</v>
       </c>
       <c r="I99" t="n">
-        <v>14.99</v>
+        <v>10.98</v>
       </c>
       <c r="J99" t="inlineStr"/>
       <c r="K99" t="inlineStr"/>
@@ -5317,18 +5317,18 @@
         <v>0</v>
       </c>
       <c r="P99" t="n">
-        <v>-2.4</v>
+        <v>1.32</v>
       </c>
       <c r="Q99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr"/>
       <c r="B100" t="n">
-        <v>1517514880</v>
+        <v>1648733962</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>KMB</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -5337,19 +5337,19 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>0.0231</v>
+        <v>0.081</v>
       </c>
       <c r="F100" s="2" t="n">
-        <v>45597.61087239583</v>
+        <v>45695.85463682871</v>
       </c>
       <c r="G100" t="n">
-        <v>409.38</v>
+        <v>129.56</v>
       </c>
       <c r="H100" t="n">
-        <v>460.45</v>
+        <v>142.67</v>
       </c>
       <c r="I100" t="n">
-        <v>9.460000000000001</v>
+        <v>10.49</v>
       </c>
       <c r="J100" t="inlineStr"/>
       <c r="K100" t="inlineStr"/>
@@ -5366,18 +5366,18 @@
         <v>0</v>
       </c>
       <c r="P100" t="n">
-        <v>1.18</v>
+        <v>1.07</v>
       </c>
       <c r="Q100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr"/>
       <c r="B101" t="n">
-        <v>1776193271</v>
+        <v>1680994777</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>BCS</t>
+          <t>APA</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -5386,19 +5386,19 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>0.6724</v>
+        <v>0.7278</v>
       </c>
       <c r="F101" s="2" t="n">
-        <v>45764.85451520833</v>
+        <v>45716.85705375</v>
       </c>
       <c r="G101" t="n">
-        <v>14.87</v>
+        <v>20.6</v>
       </c>
       <c r="H101" t="n">
-        <v>17.88</v>
+        <v>17.17</v>
       </c>
       <c r="I101" t="n">
-        <v>10</v>
+        <v>14.99</v>
       </c>
       <c r="J101" t="inlineStr"/>
       <c r="K101" t="inlineStr"/>
@@ -5415,18 +5415,18 @@
         <v>0</v>
       </c>
       <c r="P101" t="n">
-        <v>2.02</v>
+        <v>-2.49</v>
       </c>
       <c r="Q101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr"/>
       <c r="B102" t="n">
-        <v>1744916497</v>
+        <v>1517514880</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>ING</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5435,19 +5435,19 @@
         </is>
       </c>
       <c r="E102" t="n">
-        <v>1</v>
+        <v>0.0231</v>
       </c>
       <c r="F102" s="2" t="n">
-        <v>45751.74231563658</v>
+        <v>45597.61087239583</v>
       </c>
       <c r="G102" t="n">
-        <v>17.54</v>
+        <v>409.38</v>
       </c>
       <c r="H102" t="n">
-        <v>21.3</v>
+        <v>457.4</v>
       </c>
       <c r="I102" t="n">
-        <v>17.54</v>
+        <v>9.460000000000001</v>
       </c>
       <c r="J102" t="inlineStr"/>
       <c r="K102" t="inlineStr"/>
@@ -5464,18 +5464,18 @@
         <v>0</v>
       </c>
       <c r="P102" t="n">
-        <v>3.76</v>
+        <v>1.11</v>
       </c>
       <c r="Q102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr"/>
       <c r="B103" t="n">
-        <v>1825032062</v>
+        <v>1776193271</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>AGIO</t>
+          <t>BCS</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -5484,16 +5484,16 @@
         </is>
       </c>
       <c r="E103" t="n">
-        <v>0.3559</v>
+        <v>0.6724</v>
       </c>
       <c r="F103" s="2" t="n">
-        <v>45792.76080334491</v>
+        <v>45764.85451520833</v>
       </c>
       <c r="G103" t="n">
-        <v>28.09</v>
+        <v>14.87</v>
       </c>
       <c r="H103" t="n">
-        <v>30.02</v>
+        <v>17.63</v>
       </c>
       <c r="I103" t="n">
         <v>10</v>
@@ -5513,18 +5513,18 @@
         <v>0</v>
       </c>
       <c r="P103" t="n">
-        <v>0.68</v>
+        <v>1.85</v>
       </c>
       <c r="Q103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr"/>
       <c r="B104" t="n">
-        <v>1533882988</v>
+        <v>1744916497</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>BOTZ.L</t>
+          <t>ING</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -5533,19 +5533,19 @@
         </is>
       </c>
       <c r="E104" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F104" s="2" t="n">
-        <v>45609.60769543982</v>
+        <v>45751.74231563658</v>
       </c>
       <c r="G104" t="n">
-        <v>21.905</v>
+        <v>17.54</v>
       </c>
       <c r="H104" t="n">
-        <v>20.66</v>
+        <v>20.97</v>
       </c>
       <c r="I104" t="n">
-        <v>10.95</v>
+        <v>17.54</v>
       </c>
       <c r="J104" t="inlineStr"/>
       <c r="K104" t="inlineStr"/>
@@ -5562,18 +5562,18 @@
         <v>0</v>
       </c>
       <c r="P104" t="n">
-        <v>-0.62</v>
+        <v>3.43</v>
       </c>
       <c r="Q104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr"/>
       <c r="B105" t="n">
-        <v>1843477152</v>
+        <v>1825032062</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>BCS</t>
+          <t>AGIO</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -5582,19 +5582,19 @@
         </is>
       </c>
       <c r="E105" t="n">
-        <v>0.1198</v>
+        <v>0.3559</v>
       </c>
       <c r="F105" s="2" t="n">
-        <v>45804.66724922453</v>
+        <v>45792.76080334491</v>
       </c>
       <c r="G105" t="n">
-        <v>17.86</v>
+        <v>28.09</v>
       </c>
       <c r="H105" t="n">
-        <v>17.88</v>
+        <v>30.82</v>
       </c>
       <c r="I105" t="n">
-        <v>2.14</v>
+        <v>10</v>
       </c>
       <c r="J105" t="inlineStr"/>
       <c r="K105" t="inlineStr"/>
@@ -5611,18 +5611,18 @@
         <v>0</v>
       </c>
       <c r="P105" t="n">
-        <v>0</v>
+        <v>0.97</v>
       </c>
       <c r="Q105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr"/>
       <c r="B106" t="n">
-        <v>1606697510</v>
+        <v>1533882988</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>MA</t>
+          <t>BOTZ.L</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -5631,19 +5631,19 @@
         </is>
       </c>
       <c r="E106" t="n">
-        <v>0.0295</v>
+        <v>0.5</v>
       </c>
       <c r="F106" s="2" t="n">
-        <v>45667.68664726852</v>
+        <v>45609.60769543982</v>
       </c>
       <c r="G106" t="n">
-        <v>507.68</v>
+        <v>21.905</v>
       </c>
       <c r="H106" t="n">
-        <v>573.11</v>
+        <v>20.41</v>
       </c>
       <c r="I106" t="n">
-        <v>14.98</v>
+        <v>10.95</v>
       </c>
       <c r="J106" t="inlineStr"/>
       <c r="K106" t="inlineStr"/>
@@ -5660,27 +5660,45 @@
         <v>0</v>
       </c>
       <c r="P106" t="n">
-        <v>1.93</v>
+        <v>-0.74</v>
       </c>
       <c r="Q106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr"/>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="C107" t="inlineStr"/>
-      <c r="D107" t="inlineStr"/>
-      <c r="E107" t="inlineStr"/>
-      <c r="F107" t="inlineStr"/>
-      <c r="G107" t="inlineStr"/>
-      <c r="H107" t="inlineStr"/>
-      <c r="I107" t="inlineStr"/>
+      <c r="B107" t="n">
+        <v>1843477152</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>BCS</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>0.1198</v>
+      </c>
+      <c r="F107" s="2" t="n">
+        <v>45804.66724922453</v>
+      </c>
+      <c r="G107" t="n">
+        <v>17.86</v>
+      </c>
+      <c r="H107" t="n">
+        <v>17.63</v>
+      </c>
+      <c r="I107" t="n">
+        <v>2.14</v>
+      </c>
       <c r="J107" t="inlineStr"/>
       <c r="K107" t="inlineStr"/>
-      <c r="L107" t="inlineStr"/>
+      <c r="L107" t="n">
+        <v>0</v>
+      </c>
       <c r="M107" t="n">
         <v>0</v>
       </c>
@@ -5691,9 +5709,138 @@
         <v>0</v>
       </c>
       <c r="P107" t="n">
-        <v>62.79</v>
+        <v>-0.03</v>
       </c>
       <c r="Q107" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr"/>
+      <c r="B108" t="n">
+        <v>1606697510</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>MA</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>0.0295</v>
+      </c>
+      <c r="F108" s="2" t="n">
+        <v>45667.68664726852</v>
+      </c>
+      <c r="G108" t="n">
+        <v>507.68</v>
+      </c>
+      <c r="H108" t="n">
+        <v>575.73</v>
+      </c>
+      <c r="I108" t="n">
+        <v>14.98</v>
+      </c>
+      <c r="J108" t="inlineStr"/>
+      <c r="K108" t="inlineStr"/>
+      <c r="L108" t="n">
+        <v>0</v>
+      </c>
+      <c r="M108" t="n">
+        <v>0</v>
+      </c>
+      <c r="N108" t="n">
+        <v>0</v>
+      </c>
+      <c r="O108" t="n">
+        <v>0</v>
+      </c>
+      <c r="P108" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr"/>
+      <c r="B109" t="n">
+        <v>1845431561</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>AGIO</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>0.3271</v>
+      </c>
+      <c r="F109" s="2" t="n">
+        <v>45805.66210755787</v>
+      </c>
+      <c r="G109" t="n">
+        <v>30.57</v>
+      </c>
+      <c r="H109" t="n">
+        <v>30.82</v>
+      </c>
+      <c r="I109" t="n">
+        <v>10</v>
+      </c>
+      <c r="J109" t="inlineStr"/>
+      <c r="K109" t="inlineStr"/>
+      <c r="L109" t="n">
+        <v>0</v>
+      </c>
+      <c r="M109" t="n">
+        <v>0</v>
+      </c>
+      <c r="N109" t="n">
+        <v>0</v>
+      </c>
+      <c r="O109" t="n">
+        <v>0</v>
+      </c>
+      <c r="P109" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="Q109" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr"/>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr"/>
+      <c r="D110" t="inlineStr"/>
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr"/>
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr"/>
+      <c r="J110" t="inlineStr"/>
+      <c r="K110" t="inlineStr"/>
+      <c r="L110" t="inlineStr"/>
+      <c r="M110" t="n">
+        <v>0</v>
+      </c>
+      <c r="N110" t="n">
+        <v>0</v>
+      </c>
+      <c r="O110" t="n">
+        <v>0</v>
+      </c>
+      <c r="P110" t="n">
+        <v>53.71</v>
+      </c>
+      <c r="Q110" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>